<commit_message>
Added frontend and made some changes
</commit_message>
<xml_diff>
--- a/backend/LedgerWright_Reconciliation_Report.xlsx
+++ b/backend/LedgerWright_Reconciliation_Report.xlsx
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.5</v>
+        <v>0.85</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>45878</v>
@@ -1591,7 +1591,7 @@
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>'Freelancer Payment - Design' (₹5,000.00, 2025-08-09) has no corresponding entry on the other side within the statement period. No rule-based explanation fits — needs a human look.</t>
+          <t>Ledger entry for freelancer payment of 5000.0 has no matching bank statement record, requiring human review.</t>
         </is>
       </c>
     </row>
@@ -1602,7 +1602,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.5</v>
+        <v>0.85</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>45882</v>
@@ -1620,7 +1620,7 @@
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>'Petty Cash Withdrawal' (₹2,000.00, 2025-08-13) has no corresponding entry on the other side within the statement period. No rule-based explanation fits — needs a human look.</t>
+          <t>Petty cash withdrawal logged in ledger without corresponding bank transaction.</t>
         </is>
       </c>
     </row>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>45891</v>
@@ -1649,7 +1649,7 @@
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>'Consulting Fee - Q3 Advisory' (₹42,000.00, 2025-08-22) has no corresponding entry on the other side within the statement period. No rule-based explanation fits — needs a human look.</t>
+          <t>Large ledger entry for consulting fee has no bank counterpart, posing potential data entry or timing error.</t>
         </is>
       </c>
     </row>
@@ -1660,7 +1660,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.7</v>
+        <v>0.95</v>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
@@ -1678,7 +1678,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>'Bank Charge - Monthly Maintenance' (₹150.00) appears on the bank statement but has no matching ledger entry — likely a bank-initiated charge or credit never logged internally. Recommend adding this entry to the ledger.</t>
+          <t>Bank monthly maintenance fee of 150.0 appears on bank statement but was not recorded in internal ledger.</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.7</v>
+        <v>0.95</v>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
@@ -1707,7 +1707,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>'Interest Credit' (₹220.00) appears on the bank statement but has no matching ledger entry — likely a bank-initiated charge or credit never logged internally. Recommend adding this entry to the ledger.</t>
+          <t>Interest credit of 220.0 posted by bank but missing from internal ledger.</t>
         </is>
       </c>
     </row>
@@ -1718,7 +1718,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.7</v>
+        <v>0.95</v>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
@@ -1736,7 +1736,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>'Card Annual Fee' (₹499.00) appears on the bank statement but has no matching ledger entry — likely a bank-initiated charge or credit never logged internally. Recommend adding this entry to the ledger.</t>
+          <t>Card annual fee of 499.0 charged on bank statement but missing from internal ledger.</t>
         </is>
       </c>
     </row>

</xml_diff>